<commit_message>
Cambios en reportes, tipo de monedas
</commit_message>
<xml_diff>
--- a/TomaInventarioWEB/Plantillas/Plantilla_Reportes_Nuevo.xlsx
+++ b/TomaInventarioWEB/Plantillas/Plantilla_Reportes_Nuevo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\User\Desktop\Documentos\TomaDeInventario - Web\TomaInventario-GitHub\TomaInventarioWEB\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83403F56-FC06-4AB6-9A48-9F5F7A452628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F0B5E5E-C74D-49C2-AC9E-5E6A0E51E711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5490" yWindow="6015" windowWidth="19005" windowHeight="8640" xr2:uid="{341DA8A6-F758-4858-803D-93A9B3282188}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{341DA8A6-F758-4858-803D-93A9B3282188}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,13 +80,6 @@
       <b/>
       <sz val="15"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -142,19 +135,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -164,6 +150,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -173,10 +165,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -500,301 +493,301 @@
     <col min="2" max="2" width="14.5703125" style="3" customWidth="1"/>
     <col min="3" max="3" width="15.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="6" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" style="6" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="6"/>
-    <col min="10" max="10" width="15.140625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" style="6" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" style="6" customWidth="1"/>
-    <col min="13" max="13" width="16" style="6" customWidth="1"/>
-    <col min="14" max="14" width="17.28515625" style="6" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" style="6" customWidth="1"/>
-    <col min="16" max="26" width="11.42578125" style="6"/>
+    <col min="5" max="5" width="17.85546875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" style="4" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="4"/>
+    <col min="10" max="10" width="15.140625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="4" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" style="4" customWidth="1"/>
+    <col min="13" max="13" width="16" style="4" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" style="4" customWidth="1"/>
+    <col min="15" max="15" width="17.42578125" style="4" customWidth="1"/>
+    <col min="16" max="26" width="11.42578125" style="4"/>
     <col min="27" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:26" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="6"/>
+      <c r="Z1" s="6"/>
     </row>
     <row r="2" spans="2:26" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="9"/>
-      <c r="U2" s="9"/>
-      <c r="V2" s="9"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6"/>
+      <c r="Z2" s="6"/>
     </row>
     <row r="3" spans="2:26" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
-      <c r="W3" s="9"/>
-      <c r="X3" s="9"/>
-      <c r="Y3" s="9"/>
-      <c r="Z3" s="9"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
     </row>
     <row r="4" spans="2:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="15" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="9"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
-      <c r="W4" s="9"/>
-      <c r="X4" s="9"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
     </row>
     <row r="5" spans="2:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="15" t="s">
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
-      <c r="W5" s="9"/>
-      <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6"/>
+      <c r="Z5" s="6"/>
     </row>
     <row r="6" spans="2:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="15" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6"/>
+      <c r="Z6" s="6"/>
     </row>
     <row r="7" spans="2:26" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="15" t="s">
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="16"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
-      <c r="Y7" s="9"/>
-      <c r="Z7" s="9"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
     </row>
     <row r="8" spans="2:26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="6"/>
-      <c r="W8" s="6"/>
-      <c r="X8" s="6"/>
-      <c r="Y8" s="6"/>
-      <c r="Z8" s="6"/>
-    </row>
-    <row r="9" spans="2:26" s="7" customFormat="1" ht="19.5" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:26" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="8"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="4"/>
+      <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
+      <c r="Z8" s="4"/>
+    </row>
+    <row r="9" spans="2:26" s="5" customFormat="1" ht="19.5" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:26" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="16"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16"/>
+      <c r="W10" s="16"/>
+      <c r="X10" s="16"/>
+      <c r="Y10" s="16"/>
+      <c r="Z10" s="16"/>
     </row>
     <row r="11" spans="2:26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D11" s="1"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="6"/>
-      <c r="X11" s="6"/>
-      <c r="Y11" s="6"/>
-      <c r="Z11" s="6"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
+      <c r="W11" s="4"/>
+      <c r="X11" s="4"/>
+      <c r="Y11" s="4"/>
+      <c r="Z11" s="4"/>
     </row>
     <row r="12" spans="2:26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D12" s="1"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="6"/>
-      <c r="W12" s="6"/>
-      <c r="X12" s="6"/>
-      <c r="Y12" s="6"/>
-      <c r="Z12" s="6"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
+      <c r="W12" s="4"/>
+      <c r="X12" s="4"/>
+      <c r="Y12" s="4"/>
+      <c r="Z12" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>